<commit_message>
P97-3 close: gpc first drop-sync verified and wired
The drop landed and loaded all 89,386 pre-verified entries (5
id-less rows skip by rule). The first live card (aberth) exposed
two more upstream separators — "@" between sense glosses and "_"
in the plural column — fixed with the aberth row re-cut into the
fixture to pin both shapes; the re-parse updated the 30,641
affected entries and sha-skipped the rest (idempotency held).
Wired with the measured facts; the celtic desk gains its Welsh
dictionary shelf; site census/desks regenerated.
</commit_message>
<xml_diff>
--- a/test/fixtures/gpc/gpc_sample.xlsx
+++ b/test/fixtures/gpc/gpc_sample.xlsx
@@ -48,7 +48,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="36" uniqueCount="36">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="42" uniqueCount="42">
   <si>
     <t>Dangosair / Headword</t>
   </si>
@@ -156,6 +156,24 @@
   </si>
   <si>
     <t>&lt;part-of-speech&gt;&lt;pos&gt;ebd.&lt;/pos&gt; a'i ddilyn gan y tr. ml&lt;/part-of-speech&gt;</t>
+  </si>
+  <si>
+    <t>aberth</t>
+  </si>
+  <si>
+    <t>https://www.geiriadur.ac.uk/gpc/gpc.html?gpc122248</t>
+  </si>
+  <si>
+    <t>eg.b.</t>
+  </si>
+  <si>
+    <t>aberthau_aberthoedd_ebyrth</t>
+  </si>
+  <si>
+    <t>a sacrificing or offering@victim@treasure@also fig._exx. with ref. to Christ)_exx. with ref. to the Eucharist_victim (of circumstances)</t>
+  </si>
+  <si>
+    <t>&lt;part-of-speech&gt;&lt;pos&gt;eg.b.&lt;/pos&gt; ll. &lt;i&gt;aberthau&lt;/i&gt;, &lt;i&gt;aberthoedd&lt;/i&gt;, &lt;i&gt;ebyrth&lt;/i&gt;&lt;/part-of-speech&gt;</t>
   </si>
 </sst>
 </file>
@@ -785,6 +803,33 @@
         <v>35</v>
       </c>
     </row>
+    <row r="51" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A51" t="s">
+        <v>36</v>
+      </c>
+      <c r="B51" s="2" t="str">
+        <f>HYPERLINK(GPC_popeth_123[[#This Row],[URL plaen / plain URL]] GPC_popeth_123[[#This Row],[URL plaen / plain URL]])</f>
+        <v>https://www.geiriadur.ac.uk/gpc/gpc.html?gpc122248</v>
+      </c>
+      <c r="C51" t="s">
+        <v>37</v>
+      </c>
+      <c r="D51" t="s">
+        <v>12</v>
+      </c>
+      <c r="E51" t="s">
+        <v>38</v>
+      </c>
+      <c r="F51" t="s">
+        <v>39</v>
+      </c>
+      <c r="G51" t="s">
+        <v>40</v>
+      </c>
+      <c r="H51" t="s">
+        <v>41</v>
+      </c>
+    </row>
   </sheetData>
 </worksheet>
 </file>

</xml_diff>